<commit_message>
backend updates, new lines introduced
</commit_message>
<xml_diff>
--- a/backend/data/Location.xlsx
+++ b/backend/data/Location.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="2" max="3"/>
@@ -457,6 +457,11 @@
           <t>Line</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -475,6 +480,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,6 +503,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -511,6 +526,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -529,6 +549,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -547,6 +572,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -565,6 +595,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -583,6 +618,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -601,6 +641,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -619,6 +664,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -637,6 +687,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -655,6 +710,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -673,6 +733,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -691,6 +756,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -709,6 +779,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -727,6 +802,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -745,6 +825,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -763,6 +848,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -781,6 +871,11 @@
           <t>East West Corridor</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -799,6 +894,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -817,6 +917,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -835,6 +940,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -853,6 +963,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -871,6 +986,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -889,6 +1009,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -907,6 +1032,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -925,6 +1055,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -943,6 +1078,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -961,6 +1101,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -979,6 +1124,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -997,6 +1147,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1015,6 +1170,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1033,6 +1193,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1051,6 +1216,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1069,6 +1239,11 @@
           <t>North South Corridor</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1087,6 +1262,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1105,6 +1285,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1123,6 +1308,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1141,6 +1331,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1159,6 +1354,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1177,6 +1377,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1195,6 +1400,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1213,6 +1423,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1231,6 +1446,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1249,6 +1469,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1267,6 +1492,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1285,6 +1515,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1303,6 +1538,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1321,6 +1561,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1339,6 +1584,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1357,6 +1607,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1375,6 +1630,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1393,6 +1653,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1411,6 +1676,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1429,6 +1699,11 @@
           <t>Corridor-1</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1447,6 +1722,11 @@
           <t>Corridor-2</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1465,6 +1745,11 @@
           <t>Corridor-2</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1481,6 +1766,241 @@
       <c r="D58" t="inlineStr">
         <is>
           <t>Corridor-2</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Koteshwar Road</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>23.1031114</v>
+      </c>
+      <c r="C59" t="n">
+        <v>72.6021329</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Airport Corridor</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Ashram Road</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>23.0985</v>
+      </c>
+      <c r="C60" t="n">
+        <v>72.60680000000001</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Airport Corridor</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Koteshwar Prachin Mandir</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>23.09462</v>
+      </c>
+      <c r="C61" t="n">
+        <v>72.61194</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Airport Corridor</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Sabarmati River</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>23.0879</v>
+      </c>
+      <c r="C62" t="n">
+        <v>72.6181</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Airport Corridor</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Sardarnagar</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>23.08111</v>
+      </c>
+      <c r="C63" t="n">
+        <v>72.62423</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Airport Corridor</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Airport</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>23.07188</v>
+      </c>
+      <c r="C64" t="n">
+        <v>72.61976</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Airport Corridor</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Gift City</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>23.1533555</v>
+      </c>
+      <c r="C65" t="n">
+        <v>72.68555360000001</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>GIFT City Extension</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>GIFT City House</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>23.163887</v>
+      </c>
+      <c r="C66" t="n">
+        <v>72.680325</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>GIFT City Extension</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Gujarat Biotechnology University</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>23.170855</v>
+      </c>
+      <c r="C67" t="n">
+        <v>72.67346000000001</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>GIFT City Extension</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Shahpur (Gandhinagar)</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>23.1820852</v>
+      </c>
+      <c r="C68" t="n">
+        <v>72.6742387</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>GIFT City Extension</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Work in progress</t>
         </is>
       </c>
     </row>

</xml_diff>